<commit_message>
fix: change number type to integer for Excel v2
</commit_message>
<xml_diff>
--- a/definitions/shipping_rates_DMN.xlsx
+++ b/definitions/shipping_rates_DMN.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="60">
   <si>
     <t xml:space="preserve">policy</t>
   </si>
@@ -80,9 +80,6 @@
   </si>
   <si>
     <t xml:space="preserve">boolean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">number</t>
   </si>
   <si>
     <t xml:space="preserve">any</t>
@@ -657,10 +654,10 @@
         <v>19</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>18</v>
@@ -675,185 +672,185 @@
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="J4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="L4" s="0" t="s">
+      <c r="M4" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D5" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="F5" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="G5" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="G5" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" s="0" t="s">
+      <c r="J5" s="0" t="s">
         <v>35</v>
-      </c>
-      <c r="J5" s="0" t="s">
-        <v>36</v>
       </c>
       <c r="K5" s="0" t="n">
         <v>5</v>
       </c>
       <c r="L5" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="M5" s="0" t="s">
         <v>37</v>
-      </c>
-      <c r="M5" s="0" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D6" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="G6" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="H6" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="G6" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" s="0" t="s">
+      <c r="J6" s="0" t="s">
         <v>41</v>
-      </c>
-      <c r="J6" s="0" t="s">
-        <v>42</v>
       </c>
       <c r="K6" s="0" t="n">
         <v>3</v>
       </c>
       <c r="L6" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="M6" s="0" t="s">
         <v>43</v>
-      </c>
-      <c r="M6" s="0" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D7" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="G7" s="0" t="s">
+      <c r="H7" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="0" t="s">
+      <c r="I7" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="J7" s="0" t="s">
         <v>48</v>
-      </c>
-      <c r="J7" s="0" t="s">
-        <v>49</v>
       </c>
       <c r="K7" s="0" t="n">
         <v>7</v>
       </c>
       <c r="L7" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="M7" s="0" t="s">
         <v>50</v>
-      </c>
-      <c r="M7" s="0" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D8" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="F8" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="G8" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="I8" s="0" t="s">
-        <v>55</v>
-      </c>
       <c r="J8" s="0" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K8" s="0" t="n">
         <v>8</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M8" s="0" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D9" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="0" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="I9" s="0" t="s">
-        <v>58</v>
-      </c>
       <c r="J9" s="0" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K9" s="0" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="M9" s="0" t="s">
         <v>59</v>
-      </c>
-      <c r="M9" s="0" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>